<commit_message>
Corrida | SFE-ESC1 | 2026-06-17 11:32:26.504434
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ESC1_out.xlsx
+++ b/indicadores/SFE-ESC1_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="466">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Escrituras de ventas de la 1ra circunscripción de Santa Fe (Centro-Norte)</t>
+    <t xml:space="preserve">Escrituras de ventas de la 1ra circunscripción de Santa Fe</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centro-Norte de la provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">20/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1908,9 +1914,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1921,7 +1931,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1935,12 +1945,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.348828366529794</v>
+        <v>0.351277509010169</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1951,7 +1961,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1979,7 +1989,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1993,12 +2003,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.121681229295844</v>
+        <v>0.12339588833639</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2021,7 +2031,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2035,7 +2045,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2049,7 +2059,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2063,12 +2073,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00534406026960819</v>
+        <v>0.00480257631168358</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2079,7 +2089,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2093,12 +2103,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00275819101388406</v>
+        <v>0.00308779181856446</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2241,10 +2251,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2257,10 +2267,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2284,66 +2294,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>581</v>
@@ -2396,7 +2406,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>748</v>
@@ -2453,7 +2463,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>964</v>
@@ -2510,7 +2520,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>912</v>
@@ -2567,7 +2577,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>885</v>
@@ -2624,7 +2634,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>909</v>
@@ -2681,7 +2691,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>977</v>
@@ -2738,7 +2748,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>973</v>
@@ -2795,7 +2805,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1043</v>
@@ -2852,7 +2862,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1034</v>
@@ -2909,7 +2919,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1017</v>
@@ -2966,7 +2976,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1279</v>
@@ -3023,7 +3033,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>596</v>
@@ -3082,7 +3092,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>707</v>
@@ -3141,7 +3151,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>1069</v>
@@ -3200,7 +3210,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>805</v>
@@ -3259,7 +3269,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>916</v>
@@ -3318,7 +3328,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>959</v>
@@ -3377,7 +3387,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>1015</v>
@@ -3436,7 +3446,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>977</v>
@@ -3495,7 +3505,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>949</v>
@@ -3554,7 +3564,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>977</v>
@@ -3613,7 +3623,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>857</v>
@@ -3672,7 +3682,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>769</v>
@@ -3731,7 +3741,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>356</v>
@@ -3790,7 +3800,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>441</v>
@@ -3849,7 +3859,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>785</v>
@@ -3908,7 +3918,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1564</v>
@@ -3967,7 +3977,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>1357</v>
@@ -4026,7 +4036,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>898</v>
@@ -4085,7 +4095,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>974</v>
@@ -4144,7 +4154,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1175</v>
@@ -4203,7 +4213,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>1089</v>
@@ -4262,7 +4272,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>1141</v>
@@ -4321,7 +4331,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>1147</v>
@@ -4380,7 +4390,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>1481</v>
@@ -4439,7 +4449,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>706</v>
@@ -4498,7 +4508,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>847</v>
@@ -4557,7 +4567,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>988</v>
@@ -4616,7 +4626,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>970</v>
@@ -4675,7 +4685,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>1020</v>
@@ -4734,7 +4744,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>976</v>
@@ -4793,7 +4803,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>1010</v>
@@ -4852,7 +4862,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1143</v>
@@ -4911,7 +4921,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>1215</v>
@@ -4970,7 +4980,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>1340</v>
@@ -5029,7 +5039,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>1206</v>
@@ -5088,7 +5098,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>1511</v>
@@ -5147,7 +5157,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>793</v>
@@ -5206,7 +5216,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>923</v>
@@ -5265,7 +5275,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>1454</v>
@@ -5324,7 +5334,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>1366</v>
@@ -5383,7 +5393,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>1388</v>
@@ -5442,7 +5452,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>1425</v>
@@ -5501,7 +5511,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>1385</v>
@@ -5560,7 +5570,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>1372</v>
@@ -5619,7 +5629,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>1310</v>
@@ -5678,7 +5688,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>1304</v>
@@ -5737,7 +5747,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>1454</v>
@@ -5796,7 +5806,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>1517</v>
@@ -5855,7 +5865,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>817</v>
@@ -5914,7 +5924,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>983</v>
@@ -5973,7 +5983,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>1266</v>
@@ -6032,7 +6042,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>1364</v>
@@ -6091,7 +6101,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>1399</v>
@@ -6150,7 +6160,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>1300</v>
@@ -6209,7 +6219,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>1430</v>
@@ -6268,7 +6278,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>1520</v>
@@ -6327,7 +6337,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>1512</v>
@@ -6386,7 +6396,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>1419</v>
@@ -6445,7 +6455,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>1381</v>
@@ -6504,7 +6514,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>1746</v>
@@ -6563,7 +6573,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>829</v>
@@ -6622,7 +6632,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>1073</v>
@@ -6681,7 +6691,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>1450</v>
@@ -6740,7 +6750,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>1348</v>
@@ -6799,7 +6809,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>1404</v>
@@ -6858,7 +6868,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>1564</v>
@@ -6917,7 +6927,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>1279</v>
@@ -6976,7 +6986,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>1535</v>
@@ -7035,7 +7045,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>1445</v>
@@ -7094,7 +7104,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>1506</v>
@@ -7153,7 +7163,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>1405</v>
@@ -7212,7 +7222,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>1740</v>
@@ -7271,7 +7281,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>1023</v>
@@ -7330,7 +7340,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>1147</v>
@@ -7389,7 +7399,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>1576</v>
@@ -7448,7 +7458,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>1063</v>
@@ -7507,7 +7517,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>1295</v>
@@ -7566,7 +7576,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>1549</v>
@@ -7625,7 +7635,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>1324</v>
@@ -7684,7 +7694,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>1544</v>
@@ -7743,7 +7753,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>1636</v>
@@ -7802,7 +7812,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>1464</v>
@@ -7861,7 +7871,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>1192</v>
@@ -7920,7 +7930,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>2294</v>
@@ -7979,7 +7989,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>832</v>
@@ -8038,7 +8048,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>1148</v>
@@ -8097,7 +8107,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>1434</v>
@@ -8156,7 +8166,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>1484</v>
@@ -8215,7 +8225,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>1658</v>
@@ -8274,7 +8284,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>1629</v>
@@ -8333,7 +8343,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>1669</v>
@@ -8392,7 +8402,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>1380</v>
@@ -8451,7 +8461,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>1314</v>
@@ -8510,7 +8520,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>1491</v>
@@ -8569,7 +8579,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>1491</v>
@@ -8628,7 +8638,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>1632</v>
@@ -8687,7 +8697,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>655</v>
@@ -8746,7 +8756,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>903</v>
@@ -8805,7 +8815,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>1200</v>
@@ -8864,7 +8874,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>1063</v>
@@ -8923,7 +8933,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>1095</v>
@@ -8982,7 +8992,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>1196</v>
@@ -9041,7 +9051,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>1251</v>
@@ -9100,7 +9110,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>1112</v>
@@ -9159,7 +9169,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>1184</v>
@@ -9218,7 +9228,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>1254</v>
@@ -9277,7 +9287,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>1231</v>
@@ -9336,7 +9346,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>1593</v>
@@ -9395,7 +9405,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>695</v>
@@ -9454,7 +9464,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>926</v>
@@ -9513,7 +9523,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>996</v>
@@ -9572,7 +9582,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>1326</v>
@@ -9631,7 +9641,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>1223</v>
@@ -9690,7 +9700,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>1266</v>
@@ -9749,7 +9759,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>1471</v>
@@ -9808,7 +9818,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>1253</v>
@@ -9867,7 +9877,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>1457</v>
@@ -9926,7 +9936,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>1426</v>
@@ -9985,7 +9995,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>1550</v>
@@ -10044,7 +10054,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>1875</v>
@@ -10103,7 +10113,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>913</v>
@@ -10162,7 +10172,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>997</v>
@@ -10221,7 +10231,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>1298</v>
@@ -10280,7 +10290,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>1547</v>
@@ -10339,7 +10349,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>1586</v>
@@ -10398,7 +10408,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>1636</v>
@@ -10457,7 +10467,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>1753</v>
@@ -10516,7 +10526,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>1794</v>
@@ -10575,7 +10585,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>1540</v>
@@ -10634,7 +10644,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>1547</v>
@@ -10693,7 +10703,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>1725</v>
@@ -10752,7 +10762,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>2015</v>
@@ -10811,7 +10821,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>924</v>
@@ -10870,7 +10880,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>1015</v>
@@ -10929,7 +10939,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>1486</v>
@@ -10988,7 +10998,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>1289</v>
@@ -11047,7 +11057,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>1532</v>
@@ -11106,7 +11116,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>1477</v>
@@ -11165,7 +11175,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>1489</v>
@@ -11224,7 +11234,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>1611</v>
@@ -11283,7 +11293,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>1397</v>
@@ -11342,7 +11352,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>1323</v>
@@ -11401,7 +11411,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>1460</v>
@@ -11460,7 +11470,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>1716</v>
@@ -11519,7 +11529,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>842</v>
@@ -11578,7 +11588,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>851</v>
@@ -11637,7 +11647,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>1459</v>
@@ -11696,7 +11706,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>1298</v>
@@ -11755,7 +11765,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>1588</v>
@@ -11814,7 +11824,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>1441</v>
@@ -11873,7 +11883,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>1457</v>
@@ -11932,7 +11942,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>1554</v>
@@ -11991,7 +12001,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>1468</v>
@@ -12050,7 +12060,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>1542</v>
@@ -12109,7 +12119,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>1438</v>
@@ -12168,7 +12178,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>1866</v>
@@ -12227,7 +12237,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>941</v>
@@ -12286,7 +12296,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>1029</v>
@@ -12345,7 +12355,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>1262</v>
@@ -12404,7 +12414,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>1285</v>
@@ -12463,7 +12473,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>1176</v>
@@ -12522,7 +12532,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>1254</v>
@@ -12581,7 +12591,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>1505</v>
@@ -12640,7 +12650,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>1488</v>
@@ -12699,7 +12709,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>1423</v>
@@ -12758,7 +12768,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>1640</v>
@@ -12817,7 +12827,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>1255</v>
@@ -12876,7 +12886,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>1556</v>
@@ -12935,7 +12945,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>769</v>
@@ -12994,7 +13004,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>808</v>
@@ -13053,7 +13063,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>1212</v>
@@ -13112,7 +13122,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>1275</v>
@@ -13171,7 +13181,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>1168</v>
@@ -13230,7 +13240,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>1320</v>
@@ -13289,7 +13299,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>1487</v>
@@ -13348,7 +13358,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>1159</v>
@@ -13407,7 +13417,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>1301</v>
@@ -13466,7 +13476,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>1300</v>
@@ -13525,7 +13535,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>1276</v>
@@ -13584,7 +13594,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>1475</v>
@@ -13643,7 +13653,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>609</v>
@@ -13702,7 +13712,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>806</v>
@@ -13761,7 +13771,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>1089</v>
@@ -13820,7 +13830,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>1054</v>
@@ -13879,7 +13889,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>1041</v>
@@ -13938,7 +13948,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>872</v>
@@ -13997,7 +14007,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>886</v>
@@ -14056,7 +14066,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>1110</v>
@@ -14115,7 +14125,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>1045</v>
@@ -14174,7 +14184,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>1029</v>
@@ -14233,7 +14243,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>1054</v>
@@ -14292,7 +14302,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>1280</v>
@@ -14351,7 +14361,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>645</v>
@@ -14410,7 +14420,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>779</v>
@@ -14469,7 +14479,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>1025</v>
@@ -14528,7 +14538,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>1013</v>
@@ -14587,7 +14597,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>1130</v>
@@ -14646,7 +14656,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>1212</v>
@@ -14705,7 +14715,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>1125</v>
@@ -14764,7 +14774,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>1350</v>
@@ -14823,7 +14833,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>1364</v>
@@ -14882,7 +14892,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>1324</v>
@@ -14941,7 +14951,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>1340</v>
@@ -15000,7 +15010,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>1567</v>
@@ -15059,7 +15069,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>864</v>
@@ -15118,7 +15128,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>852</v>
@@ -15177,7 +15187,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>1234</v>
@@ -15236,7 +15246,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>1296</v>
@@ -15295,7 +15305,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>1305</v>
@@ -15354,7 +15364,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>1233</v>
@@ -15413,7 +15423,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>955</v>
@@ -15472,7 +15482,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>1161</v>
@@ -15531,7 +15541,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>1114</v>
@@ -15590,7 +15600,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>1138</v>
@@ -15649,7 +15659,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>1086</v>
@@ -15708,7 +15718,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>1204</v>
@@ -15767,7 +15777,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>549</v>
@@ -15826,7 +15836,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>558</v>
@@ -15885,7 +15895,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>859</v>
@@ -15944,7 +15954,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>1067</v>
@@ -16003,7 +16013,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>1058</v>
@@ -16062,7 +16072,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>939</v>
@@ -16121,7 +16131,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>899</v>
@@ -16180,7 +16190,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>957</v>
@@ -16239,7 +16249,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>931</v>
@@ -16298,7 +16308,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>978</v>
@@ -16357,7 +16367,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>1021</v>
@@ -16416,7 +16426,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>1149</v>
@@ -16475,7 +16485,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>506</v>
@@ -16534,7 +16544,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>683</v>
@@ -16593,7 +16603,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>604</v>
@@ -16652,7 +16662,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>17</v>
@@ -16711,7 +16721,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>448</v>
@@ -16770,7 +16780,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>823</v>
@@ -16829,7 +16839,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>1181</v>
@@ -16888,7 +16898,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>1231</v>
@@ -16947,7 +16957,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>1186</v>
@@ -17006,7 +17016,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>1265</v>
@@ -17065,7 +17075,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>1326</v>
@@ -17124,7 +17134,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>1512</v>
@@ -17183,7 +17193,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>775</v>
@@ -17242,7 +17252,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>947</v>
@@ -17301,7 +17311,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>1432</v>
@@ -17360,7 +17370,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>1284</v>
@@ -17419,7 +17429,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>994</v>
@@ -17478,7 +17488,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>1097</v>
@@ -17537,7 +17547,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>1395</v>
@@ -17596,7 +17606,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>1519</v>
@@ -17655,7 +17665,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>1497</v>
@@ -17714,7 +17724,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>1391</v>
@@ -17773,7 +17783,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>1463</v>
@@ -17832,7 +17842,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>1291</v>
@@ -17891,7 +17901,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>625</v>
@@ -17950,7 +17960,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>870</v>
@@ -18009,7 +18019,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>1142</v>
@@ -18068,7 +18078,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>1198</v>
@@ -18127,7 +18137,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>1107</v>
@@ -18186,7 +18196,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>1098</v>
@@ -18245,7 +18255,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>1139</v>
@@ -18304,7 +18314,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>1174</v>
@@ -18363,7 +18373,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>1221</v>
@@ -18422,7 +18432,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>1112</v>
@@ -18481,7 +18491,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>1237</v>
@@ -18540,7 +18550,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>1301</v>
@@ -18599,7 +18609,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>581</v>
@@ -18658,7 +18668,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>738</v>
@@ -18717,7 +18727,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>1048</v>
@@ -18776,7 +18786,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>904</v>
@@ -18835,7 +18845,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>821</v>
@@ -18894,7 +18904,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>826</v>
@@ -18953,7 +18963,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>991</v>
@@ -19012,7 +19022,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>1012</v>
@@ -19071,7 +19081,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>1171</v>
@@ -19130,7 +19140,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>871</v>
@@ -19189,7 +19199,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>979</v>
@@ -19248,7 +19258,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>1078</v>
@@ -19307,7 +19317,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>591</v>
@@ -19366,7 +19376,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>479</v>
@@ -19425,7 +19435,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>417</v>
@@ -19484,7 +19494,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>879</v>
@@ -19543,7 +19553,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>936</v>
@@ -19602,7 +19612,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>1011</v>
@@ -19661,7 +19671,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>1172</v>
@@ -19720,7 +19730,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>1098</v>
@@ -19779,7 +19789,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>1159</v>
@@ -19838,7 +19848,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>1276</v>
@@ -19897,7 +19907,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>1042</v>
@@ -19956,7 +19966,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>1432</v>
@@ -20015,7 +20025,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>834</v>
@@ -20074,7 +20084,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>1187</v>
@@ -20133,7 +20143,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>1226</v>
@@ -20192,7 +20202,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>1189</v>
@@ -20251,7 +20261,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>1297</v>
@@ -20310,7 +20320,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>1271</v>
@@ -20369,7 +20379,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>1512</v>
@@ -20428,7 +20438,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>1387</v>
@@ -20487,7 +20497,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>1346</v>
@@ -20546,7 +20556,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>1423</v>
@@ -20605,7 +20615,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>1369</v>
@@ -20664,7 +20674,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>1537</v>
@@ -20723,7 +20733,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>901</v>
@@ -20782,7 +20792,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>957</v>
@@ -20841,7 +20851,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>1341</v>
@@ -20900,7 +20910,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3" t="n">
@@ -20933,7 +20943,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3" t="n">
@@ -20966,7 +20976,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3" t="n">
@@ -20999,7 +21009,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3" t="n">
@@ -21032,7 +21042,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3" t="n">
@@ -21065,7 +21075,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3" t="n">
@@ -21098,7 +21108,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3" t="n">
@@ -21131,7 +21141,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3" t="n">
@@ -21164,7 +21174,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3" t="n">
@@ -21197,7 +21207,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2"/>
       <c r="C326" s="3" t="n">
@@ -21230,7 +21240,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2"/>
       <c r="C327" s="3" t="n">
@@ -21263,7 +21273,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2"/>
       <c r="C328" s="3" t="n">
@@ -21296,7 +21306,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2"/>
       <c r="C329" s="3"/>
@@ -21319,7 +21329,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2"/>
       <c r="C330" s="3"/>
@@ -21342,7 +21352,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3"/>
@@ -21365,7 +21375,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3"/>
@@ -21388,7 +21398,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3"/>
@@ -21411,7 +21421,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3"/>
@@ -21434,7 +21444,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3"/>
@@ -21457,7 +21467,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3"/>
@@ -21480,7 +21490,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3"/>
@@ -21503,7 +21513,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2"/>
       <c r="C338" s="3"/>
@@ -21526,7 +21536,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2"/>
       <c r="C339" s="3"/>
@@ -21549,7 +21559,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="3"/>
@@ -21572,7 +21582,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2"/>
       <c r="C341" s="3"/>
@@ -21595,7 +21605,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2"/>
       <c r="C342" s="3"/>
@@ -21618,7 +21628,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2"/>
       <c r="C343" s="3"/>
@@ -21641,7 +21651,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2"/>
       <c r="C344" s="3"/>
@@ -21664,7 +21674,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2"/>
       <c r="C345" s="3"/>
@@ -21687,7 +21697,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2"/>
       <c r="C346" s="3"/>
@@ -21710,7 +21720,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2"/>
       <c r="C347" s="3"/>
@@ -21733,7 +21743,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2"/>
       <c r="C348" s="3"/>
@@ -21756,7 +21766,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2"/>
       <c r="C349" s="3"/>
@@ -21779,7 +21789,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2"/>
       <c r="C350" s="3"/>
@@ -21802,7 +21812,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2"/>
       <c r="C351" s="3"/>
@@ -21825,7 +21835,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2"/>
       <c r="C352" s="3"/>
@@ -21848,7 +21858,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2"/>
       <c r="C353" s="3"/>
@@ -21871,7 +21881,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2"/>
       <c r="C354" s="3"/>
@@ -21894,7 +21904,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2"/>
       <c r="C355" s="3"/>
@@ -21917,7 +21927,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2"/>
       <c r="C356" s="3"/>
@@ -21940,7 +21950,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2"/>
       <c r="C357" s="3"/>
@@ -21963,7 +21973,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2"/>
       <c r="C358" s="3"/>
@@ -21986,7 +21996,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2"/>
       <c r="C359" s="3"/>
@@ -22009,7 +22019,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2"/>
       <c r="C360" s="3"/>
@@ -22032,7 +22042,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2"/>
       <c r="C361" s="3"/>
@@ -22055,7 +22065,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2"/>
       <c r="C362" s="3"/>
@@ -22078,7 +22088,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2"/>
       <c r="C363" s="3"/>
@@ -22101,7 +22111,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2"/>
       <c r="C364" s="3"/>
@@ -22124,7 +22134,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2"/>
       <c r="C365" s="3"/>
@@ -22147,7 +22157,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2"/>
       <c r="C366" s="3"/>
@@ -22170,7 +22180,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3"/>
@@ -22193,7 +22203,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3"/>
@@ -22216,7 +22226,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3"/>
@@ -22239,7 +22249,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3"/>
@@ -22262,7 +22272,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3"/>
@@ -22285,7 +22295,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3"/>
@@ -22308,7 +22318,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3"/>
@@ -22342,97 +22352,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -22456,7 +22466,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -22466,160 +22476,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0948358566173715</v>
+        <v>0.0939841249748311</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.115612672336015</v>
+        <v>0.114764857664914</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.110936957224675</v>
+        <v>0.110658258774319</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.125937590371093</v>
+        <v>0.126215872716938</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.116653780994609</v>
+        <v>0.116833723416553</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.1387545482265</v>
+        <v>0.137945602498689</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.221335035862065</v>
+        <v>0.220161923300739</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.277601630306613</v>
+        <v>0.277576772770983</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.329065049043526</v>
+        <v>0.330680061656956</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.348828366529794</v>
+        <v>0.351277509010169</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.269647650412812</v>
+        <v>0.271759874625759</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.180080016826278</v>
+        <v>0.180790891661677</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.137553001152443</v>
+        <v>0.137136498113735</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.104395501663895</v>
+        <v>0.104148095060044</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0478362537664721</v>
+        <v>0.0475379057711405</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0296364663156039</v>
+        <v>-0.0292736516295028</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0862967603352597</v>
+        <v>-0.0839731440243371</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.107210245812731</v>
+        <v>-0.104573357615804</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.133683606997915</v>
+        <v>-0.132376581468945</v>
       </c>
     </row>
     <row r="24">

</xml_diff>